<commit_message>
Update production calculation logic and display results in the main production notebook
</commit_message>
<xml_diff>
--- a/ข้อ2.xlsx
+++ b/ข้อ2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Product_AMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B63713A-FC6B-4A7D-94DF-395DB604519F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D39A3B97-BCDD-4BCE-9567-309F7EDD1B79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3E6D1783-A657-4040-8780-286ED815531D}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{3E6D1783-A657-4040-8780-286ED815531D}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="37">
   <si>
     <t>เดือน</t>
   </si>
@@ -145,6 +145,12 @@
   </si>
   <si>
     <t>ว่างงาน</t>
+  </si>
+  <si>
+    <t>ค่าว่างงาน</t>
+  </si>
+  <si>
+    <t>ค่าของ</t>
   </si>
 </sst>
 </file>
@@ -524,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B13E4804-BD06-4C6C-BF26-5931CE160AEA}">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="9.59765625" bestFit="1" customWidth="1"/>
@@ -631,7 +637,7 @@
         <v>10</v>
       </c>
       <c r="B6">
-        <v>50</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -661,7 +667,7 @@
       </c>
       <c r="B8">
         <f>IF(B7&gt;$B$6, B7-$B$6, 0)</f>
-        <v>550</v>
+        <v>100</v>
       </c>
       <c r="C8">
         <f>IF(C7&gt;B7, C7-B7, 0)</f>
@@ -718,110 +724,177 @@
         <v>0</v>
       </c>
     </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11">
+        <f>IF(B7&gt;B4, 0, B4-B7)</f>
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <f>IF(C7&gt;C4, 0, C4-C7)</f>
+        <v>300</v>
+      </c>
+      <c r="D11">
+        <f>IF(D7&gt;D4, 0, D4-D7)</f>
+        <v>100</v>
+      </c>
+      <c r="E11">
+        <f>IF(E7&gt;E4, 0, E4-E7)</f>
+        <v>0</v>
+      </c>
+    </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12">
+        <f>IF(B$7&gt;B$4,(B7-B4),0)</f>
+        <v>140</v>
+      </c>
+      <c r="C12">
+        <f t="shared" ref="C12:E12" si="5">IF(C$7&gt;C$4,(C7-C4),0)</f>
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="5"/>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13">
+        <f>(B3*0.5)*1600</f>
+        <v>32000</v>
+      </c>
+      <c r="C13">
+        <f t="shared" ref="C13:E13" si="6">(C3*0.5)*1600</f>
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <f>SUM(B13:E13)</f>
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>16</v>
       </c>
-      <c r="B12">
+      <c r="B14">
         <f>IF(B$7&gt;B$4,B$4*40*100,B$7*40*100)</f>
         <v>1840000</v>
       </c>
-      <c r="C12">
-        <f t="shared" ref="C12:E12" si="5">IF(C$7&gt;C$4,C$4*40*100,C$7*40*100)</f>
+      <c r="C14">
+        <f t="shared" ref="C14:E14" si="7">IF(C$7&gt;C$4,C$4*40*100,C$7*40*100)</f>
         <v>2400000</v>
       </c>
-      <c r="D12">
-        <f t="shared" si="5"/>
+      <c r="D14">
+        <f t="shared" si="7"/>
         <v>2400000</v>
       </c>
-      <c r="E12">
-        <f t="shared" si="5"/>
+      <c r="E14">
+        <f t="shared" si="7"/>
         <v>1200000</v>
       </c>
-      <c r="F12">
-        <f>SUM(B12:E12)</f>
+      <c r="F14">
+        <f>SUM(B14:E14)</f>
         <v>7840000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B13">
-        <f>IF(B$7&gt;B$4,0,(B$4-B$7)*60*100)</f>
-        <v>0</v>
-      </c>
-      <c r="C13">
-        <f t="shared" ref="C13:E13" si="6">IF(C$7&gt;C$4,0,(C$4-C$7)*60*100)</f>
-        <v>1800000</v>
-      </c>
-      <c r="D13">
-        <f t="shared" si="6"/>
-        <v>600000</v>
-      </c>
-      <c r="E13">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F13">
-        <f t="shared" ref="F13:F14" si="7">SUM(B13:E13)</f>
-        <v>2400000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14">
-        <f>IF(B$7&gt;B$4,(B7-B4)*30*100,0)</f>
-        <v>420000</v>
-      </c>
-      <c r="C14">
-        <f t="shared" ref="C14:E14" si="8">IF(C$7&gt;C$4,(C7-C4)*30*100,0)</f>
-        <v>0</v>
-      </c>
-      <c r="D14">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="E14">
-        <f t="shared" si="8"/>
-        <v>900000</v>
-      </c>
-      <c r="F14">
-        <f t="shared" si="7"/>
-        <v>1320000</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15">
+        <f>B11*100*60</f>
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <f t="shared" ref="C15:E15" si="8">C11*100*60</f>
+        <v>1800000</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="8"/>
+        <v>600000</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <f t="shared" ref="F15:F16" si="9">SUM(B15:E15)</f>
+        <v>2400000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16">
+        <f>B12*30*100</f>
+        <v>420000</v>
+      </c>
+      <c r="C16">
+        <f t="shared" ref="C16:E16" si="10">C12*30*100</f>
+        <v>0</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="10"/>
+        <v>900000</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="9"/>
+        <v>1320000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>33</v>
       </c>
-      <c r="B15">
+      <c r="B17">
         <f>B8*1000</f>
-        <v>550000</v>
-      </c>
-      <c r="C15">
+        <v>100000</v>
+      </c>
+      <c r="C17">
         <f>C8*2000</f>
         <v>0</v>
       </c>
-      <c r="D15">
+      <c r="D17">
         <f>D8*2000</f>
         <v>0</v>
       </c>
-      <c r="E15">
+      <c r="E17">
         <f>E8*2000</f>
         <v>0</v>
       </c>
-      <c r="F15">
-        <f>SUM(B15:E15)</f>
-        <v>550000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F16">
-        <f>SUM(F12:F15)</f>
-        <v>12110000</v>
+      <c r="F17">
+        <f>SUM(B17:E17)</f>
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F18">
+        <f>SUM(F13:F17)</f>
+        <v>11692000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add new Excel files and update existing ones
- Created a new Excel file: ข้อ1.xlsx
- Updated existing Excel file: 𝑢𝑢𝑢2.xlsx with binary differences
</commit_message>
<xml_diff>
--- a/ข้อ2.xlsx
+++ b/ข้อ2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Product_AMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D39A3B97-BCDD-4BCE-9567-309F7EDD1B79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5C3FF3F-D92A-4F2E-B3FC-26110CED61B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{3E6D1783-A657-4040-8780-286ED815531D}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{3E6D1783-A657-4040-8780-286ED815531D}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>

</xml_diff>